<commit_message>
Incorpora directorio de establecimientos en Mensajes
</commit_message>
<xml_diff>
--- a/resources/templates/plantilla-carga-establecimientos.xlsx
+++ b/resources/templates/plantilla-carga-establecimientos.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATRIZ ESTAB" sheetId="1" r:id="R44a113de10924231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCCIONES" sheetId="2" r:id="R88560aa58ad34769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MATRIZ ESTAB" sheetId="1" r:id="R78e05c3ee5424e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCCIONES" sheetId="2" r:id="R1303f36dc76948ea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -123,7 +123,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -155,8 +155,13 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFBFBF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="16">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -296,11 +301,25 @@
         <x:color rgb="FF000000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFBFBFBF"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0"/>
@@ -378,6 +397,22 @@
     <x:xf numFmtId="0" fontId="8" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -672,6 +707,8 @@
     <x:col min="16" max="16" width="14" customWidth="1"/>
     <x:col min="17" max="17" width="14" customWidth="1"/>
     <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="25" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -739,6 +776,12 @@
       </x:c>
       <x:c r="R1" s="32" t="str">
         <x:v>MATRICULA_TOTAL</x:v>
+      </x:c>
+      <x:c r="S1" s="41" t="str">
+        <x:v>DIRECTOR_NOMBRE</x:v>
+      </x:c>
+      <x:c r="T1" s="41" t="str">
+        <x:v>DIRECTOR_CONTACTO</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15.75" customHeight="1">
@@ -788,6 +831,8 @@
       <x:c r="P2" s="22" t="n"/>
       <x:c r="Q2" s="22" t="n"/>
       <x:c r="R2" s="36"/>
+      <x:c r="S2" s="42"/>
+      <x:c r="T2" s="42"/>
     </x:row>
     <x:row r="3">
       <x:c r="R3" s="26"/>
@@ -3806,7 +3851,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb42f0ffa235e47f2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3863cf28694b0e"/>
 </x:worksheet>
 </file>
 
@@ -3814,7 +3859,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" customWidth="1"/>
+    <x:col min="1" max="1" width="68" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" customWidth="1"/>
     <x:col min="3" max="3" width="12" customWidth="1"/>
     <x:col min="4" max="4" width="24" customWidth="1"/>
@@ -4042,6 +4087,16 @@
         <x:v>20</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="37" t="str">
+        <x:v>5. DIRECTOR_NOMBRE y DIRECTOR_CONTACTO son opcionales.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="37" t="str">
+        <x:v>6. DIRECTOR_CONTACTO puede contener correo, teléfono o ambos.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>